<commit_message>
fix(store): support historical issued migration and auth guard refresh
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/issued-migration/issued_items_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/issued-migration/issued_items_migration_template.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="item_type_options">'_validations'!$A$1:$A$2</definedName>
-    <definedName name="category_name_options">'_validations'!$B$1:$B$49</definedName>
+    <definedName name="category_name_options">'_validations'!$B$1:$B$251</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="317">
   <si>
     <t>Field</t>
   </si>
@@ -47,7 +47,13 @@
     <t>employee_emp_id</t>
   </si>
   <si>
-    <t>Mandatory on first row of employee block; must exist in Employee table.</t>
+    <t>Required. Issued migration currently supports employee-based issuance only. Keep employee fields blank for continuation rows of the same employee.</t>
+  </si>
+  <si>
+    <t>Current scope</t>
+  </si>
+  <si>
+    <t>Do not provide division/vehicle/custodian values in this migration. Historical issued data is imported in employee format only.</t>
   </si>
   <si>
     <t>category_name</t>
@@ -86,6 +92,12 @@
     <t>For item_type=Asset: serial_number is preferred. asset_tag is optional (auto-generated if blank for new assets).</t>
   </si>
   <si>
+    <t>Historical asset rows without serial number</t>
+  </si>
+  <si>
+    <t>For old register data only: if serial_number and asset_tag are both blank, give the cumulative asset quantity in one row. The system will create that many issued asset records with migration placeholders internally.</t>
+  </si>
+  <si>
     <t>Consumable rows</t>
   </si>
   <si>
@@ -194,19 +206,13 @@
     <t>Personnel &amp; Administrative Division</t>
   </si>
   <si>
-    <t>Desktop</t>
-  </si>
-  <si>
-    <t>Desktop Workstation</t>
-  </si>
-  <si>
-    <t>SN-DT-0007</t>
+    <t>Laptops i5 512GB SSD 8GB RAM</t>
   </si>
   <si>
     <t>2026-02-11</t>
   </si>
   <si>
-    <t>New employee block starts</t>
+    <t>Historical asset issue without serial numbers</t>
   </si>
   <si>
     <t>LEGACY-ISSUE-EMP102-01</t>
@@ -218,54 +224,360 @@
     <t>A3 Paper Rim</t>
   </si>
   <si>
+    <t>A4 Paper Rim</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>Acid</t>
+  </si>
+  <si>
+    <t>Adapter</t>
+  </si>
+  <si>
+    <t>Adhesive Tape</t>
+  </si>
+  <si>
+    <t>Agarbati</t>
+  </si>
+  <si>
+    <t>All Pin</t>
+  </si>
+  <si>
+    <t>Almirah</t>
+  </si>
+  <si>
     <t>Attendance Register</t>
   </si>
   <si>
+    <t>Attendance register</t>
+  </si>
+  <si>
+    <t>Attendance Register (Small)</t>
+  </si>
+  <si>
+    <t>Ball Pen Achiever</t>
+  </si>
+  <si>
+    <t>Ball Pen Black</t>
+  </si>
+  <si>
+    <t>Ball Pen Blue</t>
+  </si>
+  <si>
+    <t>Ball Pen Green</t>
+  </si>
+  <si>
+    <t>Ball Pen Red</t>
+  </si>
+  <si>
+    <t>Ball Pen Uniball</t>
+  </si>
+  <si>
+    <t>Ball Pen V5</t>
+  </si>
+  <si>
+    <t>Bell</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Binder Clip  32MM</t>
+  </si>
+  <si>
+    <t>Binder Clip 25 MM</t>
+  </si>
+  <si>
+    <t>Binding Machine</t>
+  </si>
+  <si>
+    <t>Black Ball Pen</t>
+  </si>
+  <si>
     <t>Black Gel Pen</t>
   </si>
   <si>
+    <t>Black Hit</t>
+  </si>
+  <si>
+    <t>Blue Ball Pen</t>
+  </si>
+  <si>
     <t>Blue Gel Pen</t>
   </si>
   <si>
+    <t>Board Marker</t>
+  </si>
+  <si>
+    <t>Boki Chok Pump</t>
+  </si>
+  <si>
+    <t>Brown Khaki Tape</t>
+  </si>
+  <si>
+    <t>Brush Toilet</t>
+  </si>
+  <si>
+    <t>Button Folder F/S</t>
+  </si>
+  <si>
+    <t>Cables</t>
+  </si>
+  <si>
+    <t>Calculator</t>
+  </si>
+  <si>
+    <t>Camera</t>
+  </si>
+  <si>
+    <t>Candle</t>
+  </si>
+  <si>
+    <t>Carbon Paper</t>
+  </si>
+  <si>
+    <t>Cartridge</t>
+  </si>
+  <si>
+    <t>CD / OHP Marker</t>
+  </si>
+  <si>
     <t>Ceiling Fan</t>
   </si>
   <si>
+    <t>Cello Tape 1/2”</t>
+  </si>
+  <si>
+    <t>Cello Tape 2” (Big)</t>
+  </si>
+  <si>
+    <t>Chair</t>
+  </si>
+  <si>
+    <t>Chowk 15watt</t>
+  </si>
+  <si>
+    <t>Chowk Electronic 36 Watt</t>
+  </si>
+  <si>
+    <t>Clutch Pencil</t>
+  </si>
+  <si>
+    <t>CMOS Cell</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Cooler</t>
+  </si>
+  <si>
+    <t>Cube Sanitary</t>
+  </si>
+  <si>
+    <t>Cup</t>
+  </si>
+  <si>
+    <t>Cutter</t>
+  </si>
+  <si>
+    <t>Dak Pad</t>
+  </si>
+  <si>
+    <t>Damper</t>
+  </si>
+  <si>
     <t>Desktop Computer i5</t>
   </si>
   <si>
     <t>Desktop Computer i7</t>
   </si>
   <si>
+    <t>Dettol pump 200ML</t>
+  </si>
+  <si>
+    <t>Diesel</t>
+  </si>
+  <si>
+    <t>Digital Podium</t>
+  </si>
+  <si>
+    <t>Dispatch Register</t>
+  </si>
+  <si>
     <t>Double Punch</t>
   </si>
   <si>
+    <t>Double Punch ( Big)</t>
+  </si>
+  <si>
+    <t>Double Punch (Small)</t>
+  </si>
+  <si>
+    <t>Drill Bits</t>
+  </si>
+  <si>
+    <t>Dry Mop Set</t>
+  </si>
+  <si>
+    <t>Dustbin Plastic (Small) with cover</t>
+  </si>
+  <si>
+    <t>Dustbin without cover</t>
+  </si>
+  <si>
+    <t>Duster</t>
+  </si>
+  <si>
+    <t>Electrical Kettle</t>
+  </si>
+  <si>
     <t>Emergency Office Purchase</t>
   </si>
   <si>
+    <t>Engagement stand</t>
+  </si>
+  <si>
+    <t>Envelop 10X145(Yellow F/Size)</t>
+  </si>
+  <si>
+    <t>Envelop 11x5 (Plain/  Without Window)</t>
+  </si>
+  <si>
+    <t>Envelop Plain(6x3)</t>
+  </si>
+  <si>
+    <t>Envelop Window  (11x4 /11x5)</t>
+  </si>
+  <si>
+    <t>Envelope Khaki A4 Size</t>
+  </si>
+  <si>
+    <t>ESI Register</t>
+  </si>
+  <si>
     <t>Exhaust Fan</t>
   </si>
   <si>
+    <t>Extension Board</t>
+  </si>
+  <si>
+    <t>External Hard disk</t>
+  </si>
+  <si>
     <t>External Hard Disk 1TB</t>
   </si>
   <si>
+    <t>Fan Regulator</t>
+  </si>
+  <si>
+    <t>Fevi Gum  (Small)</t>
+  </si>
+  <si>
+    <t>File Cover Khaki</t>
+  </si>
+  <si>
+    <t>File Cover Yellow</t>
+  </si>
+  <si>
+    <t>File Flapper</t>
+  </si>
+  <si>
+    <t>File Tag (Green)</t>
+  </si>
+  <si>
+    <t>Finger print scanner</t>
+  </si>
+  <si>
     <t>Floor Cleaner</t>
   </si>
   <si>
+    <t>Fluid / Correction Pen</t>
+  </si>
+  <si>
+    <t>Fountain Pen(Blue)</t>
+  </si>
+  <si>
+    <t>Garbage Bag(Big)</t>
+  </si>
+  <si>
+    <t>Garbage Bag(small)</t>
+  </si>
+  <si>
     <t>Garden Shovel</t>
   </si>
   <si>
+    <t>Gate pass Book</t>
+  </si>
+  <si>
+    <t>Glass</t>
+  </si>
+  <si>
+    <t>Gloves plastic</t>
+  </si>
+  <si>
+    <t>Glustic</t>
+  </si>
+  <si>
+    <t>Godrej air poket</t>
+  </si>
+  <si>
+    <t>Gum Bottle</t>
+  </si>
+  <si>
     <t>Hand Wash Liquid</t>
   </si>
   <si>
+    <t>Harpic (Blue)</t>
+  </si>
+  <si>
+    <t>Harpic (Red)</t>
+  </si>
+  <si>
+    <t>Hi-Lighter</t>
+  </si>
+  <si>
     <t>Highlighter Pen</t>
   </si>
   <si>
+    <t>Hot Case</t>
+  </si>
+  <si>
+    <t>Induction</t>
+  </si>
+  <si>
+    <t>Ink Pilot Pen</t>
+  </si>
+  <si>
+    <t>Ink Stamps</t>
+  </si>
+  <si>
     <t>Inkjet Cartridge Black</t>
   </si>
   <si>
     <t>Inkjet Cartridge Color</t>
   </si>
   <si>
+    <t>Izyol 500ML</t>
+  </si>
+  <si>
+    <t>Jharu (Soft Broom)</t>
+  </si>
+  <si>
+    <t>Jharu stick(Bans)</t>
+  </si>
+  <si>
+    <t>Jug</t>
+  </si>
+  <si>
+    <t>Key Board</t>
+  </si>
+  <si>
+    <t>Ladder</t>
+  </si>
+  <si>
     <t>Laptop i5 8GB 512GB</t>
   </si>
   <si>
@@ -275,9 +587,60 @@
     <t>LED Monitor 24 Inch</t>
   </si>
   <si>
+    <t>LED Pannel Light</t>
+  </si>
+  <si>
+    <t>LED T.V</t>
+  </si>
+  <si>
     <t>LED TV 43 Inch</t>
   </si>
   <si>
+    <t>Legal Noting Rim</t>
+  </si>
+  <si>
+    <t>Legal Rim</t>
+  </si>
+  <si>
+    <t>Lifebouy soap</t>
+  </si>
+  <si>
+    <t>Liquid Soap</t>
+  </si>
+  <si>
+    <t>Lock</t>
+  </si>
+  <si>
+    <t>Log Book</t>
+  </si>
+  <si>
+    <t>M fold tissue</t>
+  </si>
+  <si>
+    <t>MCB Box</t>
+  </si>
+  <si>
+    <t>Mobile Phone</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>MRN Book</t>
+  </si>
+  <si>
+    <t>Name Plates</t>
+  </si>
+  <si>
+    <t>Nirma surf powder</t>
+  </si>
+  <si>
+    <t>Noting Sheet</t>
+  </si>
+  <si>
+    <t>Odonil</t>
+  </si>
+  <si>
     <t>Office Car Diesel</t>
   </si>
   <si>
@@ -293,57 +656,258 @@
     <t>Office Notebook</t>
   </si>
   <si>
+    <t>Oven</t>
+  </si>
+  <si>
+    <t>Paper Weight</t>
+  </si>
+  <si>
+    <t>Pen drive</t>
+  </si>
+  <si>
     <t>Pen Drive 64GB</t>
   </si>
   <si>
+    <t>Pen stand</t>
+  </si>
+  <si>
+    <t>Pencil Cell</t>
+  </si>
+  <si>
+    <t>Pencil Ordinary</t>
+  </si>
+  <si>
+    <t>Peon Book / Acknowledgement Book</t>
+  </si>
+  <si>
     <t>Permanent Marker</t>
   </si>
   <si>
     <t>Phenyl Cleaner</t>
   </si>
   <si>
+    <t>Photocopier</t>
+  </si>
+  <si>
+    <t>Photostat paper A4 Size</t>
+  </si>
+  <si>
+    <t>Photostat Paper F/S</t>
+  </si>
+  <si>
+    <t>Phynol</t>
+  </si>
+  <si>
     <t>Pilot Blue Pen</t>
   </si>
   <si>
+    <t>Pilot Pen V7</t>
+  </si>
+  <si>
+    <t>Pin Cushion</t>
+  </si>
+  <si>
+    <t>Pochha  Simple</t>
+  </si>
+  <si>
+    <t>Poker</t>
+  </si>
+  <si>
+    <t>Pot</t>
+  </si>
+  <si>
+    <t>Printer</t>
+  </si>
+  <si>
     <t>Projector</t>
   </si>
   <si>
+    <t>PVC Pipes</t>
+  </si>
+  <si>
+    <t>Receipt Register</t>
+  </si>
+  <si>
+    <t>Refill Ordinary</t>
+  </si>
+  <si>
+    <t>Refrigerator</t>
+  </si>
+  <si>
+    <t>Register 04 Q</t>
+  </si>
+  <si>
+    <t>Register 2Q</t>
+  </si>
+  <si>
     <t>Ring Binder File</t>
   </si>
   <si>
+    <t>Room freshner</t>
+  </si>
+  <si>
+    <t>Room Heater</t>
+  </si>
+  <si>
+    <t>Router</t>
+  </si>
+  <si>
+    <t>Rubber Band</t>
+  </si>
+  <si>
+    <t>Rubber Ordinary</t>
+  </si>
+  <si>
+    <t>Scale Plastic</t>
+  </si>
+  <si>
+    <t>Scale Steel</t>
+  </si>
+  <si>
+    <t>Scanner</t>
+  </si>
+  <si>
+    <t>Scissor</t>
+  </si>
+  <si>
+    <t>Scotch brite</t>
+  </si>
+  <si>
+    <t>Screw Driver</t>
+  </si>
+  <si>
+    <t>Server</t>
+  </si>
+  <si>
+    <t>Service Book</t>
+  </si>
+  <si>
+    <t>Sharpner</t>
+  </si>
+  <si>
     <t>Single Punch</t>
   </si>
   <si>
+    <t>Sketch Pen</t>
+  </si>
+  <si>
+    <t>Slip Pad (Ordinary)</t>
+  </si>
+  <si>
+    <t>Soap Rin /Lux</t>
+  </si>
+  <si>
+    <t>Socket</t>
+  </si>
+  <si>
+    <t>Socket 15 amp</t>
+  </si>
+  <si>
+    <t>Sofa</t>
+  </si>
+  <si>
+    <t>Spiral pad</t>
+  </si>
+  <si>
     <t>Spring File</t>
   </si>
   <si>
     <t>SSD 512GB</t>
   </si>
   <si>
+    <t>Stamp for CO Proc</t>
+  </si>
+  <si>
+    <t>Stamp Pad</t>
+  </si>
+  <si>
+    <t>Stamp Pad Ink</t>
+  </si>
+  <si>
+    <t>Standing Fan</t>
+  </si>
+  <si>
     <t>Stapler</t>
   </si>
   <si>
-    <t>Stapler Pin Big</t>
+    <t>Stapler Big</t>
+  </si>
+  <si>
+    <t>Stapler pin Big</t>
   </si>
   <si>
     <t>Stapler Pin Small</t>
   </si>
   <si>
+    <t>Stapler Small</t>
+  </si>
+  <si>
     <t>Steel Almirah</t>
   </si>
   <si>
+    <t>Stick Note Pad (Yellow)</t>
+  </si>
+  <si>
     <t>Stock Register</t>
   </si>
   <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Tablets</t>
+  </si>
+  <si>
+    <t>Telephone Register</t>
+  </si>
+  <si>
+    <t>Telephone Set</t>
+  </si>
+  <si>
+    <t>Test Category 1</t>
+  </si>
+  <si>
+    <t>Test Cateogry 2</t>
+  </si>
+  <si>
+    <t>Toilet Paper roll</t>
+  </si>
+  <si>
+    <t>Toner</t>
+  </si>
+  <si>
+    <t>Tonner General</t>
+  </si>
+  <si>
+    <t>Tray</t>
+  </si>
+  <si>
+    <t>U Clip</t>
+  </si>
+  <si>
     <t>U Clip Box</t>
   </si>
   <si>
+    <t>Umbrella</t>
+  </si>
+  <si>
     <t>Uniball black Pen</t>
   </si>
   <si>
     <t>Uniball blue Pen</t>
   </si>
   <si>
+    <t>UPS</t>
+  </si>
+  <si>
+    <t>Urinal Cube</t>
+  </si>
+  <si>
+    <t>Urnal screen(Jali)</t>
+  </si>
+  <si>
     <t>V5 blue Pen</t>
   </si>
   <si>
@@ -353,13 +917,58 @@
     <t>V7 Green Pen</t>
   </si>
   <si>
+    <t>Vim Bar</t>
+  </si>
+  <si>
+    <t>Vim Liquid</t>
+  </si>
+  <si>
+    <t>Visitor Card Album</t>
+  </si>
+  <si>
     <t>Visitor Chair</t>
   </si>
   <si>
+    <t>Visitor Slip</t>
+  </si>
+  <si>
+    <t>Wall Clock</t>
+  </si>
+  <si>
+    <t>Wall Fan</t>
+  </si>
+  <si>
+    <t>Water Bottle</t>
+  </si>
+  <si>
+    <t>Water dispenser</t>
+  </si>
+  <si>
     <t>Water Hose Pipe</t>
   </si>
   <si>
+    <t>Weighing Machine</t>
+  </si>
+  <si>
+    <t>Wet Mop Refil</t>
+  </si>
+  <si>
+    <t>Wet Mop Set</t>
+  </si>
+  <si>
+    <t>White Tag</t>
+  </si>
+  <si>
+    <t>Wiper Small</t>
+  </si>
+  <si>
+    <t>Wire</t>
+  </si>
+  <si>
     <t>Wooden Cabinet</t>
+  </si>
+  <si>
+    <t>Yellow envelop A4 Size</t>
   </si>
 </sst>
 </file>
@@ -766,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -885,8 +1494,24 @@
         <v>27</v>
       </c>
     </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -917,58 +1542,58 @@
   <sheetData>
     <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -979,52 +1604,52 @@
         <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="O2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="P2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -1032,55 +1657,55 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="L3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N3">
         <v>5</v>
       </c>
       <c r="O3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="P3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="R3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1091,52 +1716,52 @@
         <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L4" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
-      </c>
-      <c r="N4" t="s">
-        <v>43</v>
+        <v>47</v>
+      </c>
+      <c r="N4">
+        <v>30</v>
       </c>
       <c r="O4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="P4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="Q4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="R4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="5:6" x14ac:dyDescent="0.25"/>
@@ -6158,7 +6783,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B252"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -6167,10 +6792,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -6178,7 +6803,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -6186,7 +6811,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -6194,7 +6819,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -6202,7 +6827,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -6210,7 +6835,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -6218,7 +6843,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -6226,7 +6851,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -6234,7 +6859,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -6242,7 +6867,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -6250,7 +6875,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -6258,7 +6883,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -6266,7 +6891,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -6274,7 +6899,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -6282,7 +6907,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -6290,7 +6915,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -6298,7 +6923,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -6306,7 +6931,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -6314,7 +6939,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -6322,7 +6947,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -6330,7 +6955,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -6338,7 +6963,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -6346,7 +6971,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -6354,7 +6979,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -6362,7 +6987,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -6370,7 +6995,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -6378,7 +7003,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -6386,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -6394,7 +7019,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -6402,7 +7027,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -6410,7 +7035,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -6418,7 +7043,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -6426,7 +7051,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -6434,7 +7059,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -6442,7 +7067,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -6450,7 +7075,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -6458,7 +7083,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -6466,7 +7091,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -6474,7 +7099,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -6482,7 +7107,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -6490,7 +7115,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -6498,7 +7123,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -6506,7 +7131,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -6514,7 +7139,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -6522,7 +7147,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -6530,7 +7155,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -6538,7 +7163,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -6546,7 +7171,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -6554,7 +7179,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -6562,11 +7187,1627 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114">
         <v>113</v>
       </c>
+      <c r="B114" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>201</v>
+      </c>
+      <c r="B202" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>202</v>
+      </c>
+      <c r="B203" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>203</v>
+      </c>
+      <c r="B204" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>204</v>
+      </c>
+      <c r="B205" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>222</v>
+      </c>
+      <c r="B223" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>223</v>
+      </c>
+      <c r="B224" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>224</v>
+      </c>
+      <c r="B225" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>227</v>
+      </c>
+      <c r="B228" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>228</v>
+      </c>
+      <c r="B229" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>229</v>
+      </c>
+      <c r="B230" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>230</v>
+      </c>
+      <c r="B231" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>231</v>
+      </c>
+      <c r="B232" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>232</v>
+      </c>
+      <c r="B233" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>233</v>
+      </c>
+      <c r="B234" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>234</v>
+      </c>
+      <c r="B235" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>235</v>
+      </c>
+      <c r="B236" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>236</v>
+      </c>
+      <c r="B237" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>237</v>
+      </c>
+      <c r="B238" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>238</v>
+      </c>
+      <c r="B239" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A240">
+        <v>239</v>
+      </c>
+      <c r="B240" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>240</v>
+      </c>
+      <c r="B241" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>241</v>
+      </c>
+      <c r="B242" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>242</v>
+      </c>
+      <c r="B243" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>243</v>
+      </c>
+      <c r="B244" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>244</v>
+      </c>
+      <c r="B245" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>245</v>
+      </c>
+      <c r="B246" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>246</v>
+      </c>
+      <c r="B247" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>247</v>
+      </c>
+      <c r="B248" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>248</v>
+      </c>
+      <c r="B249" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>249</v>
+      </c>
+      <c r="B250" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>250</v>
+      </c>
+      <c r="B251" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>251</v>
+      </c>
+      <c r="B252" t="s">
+        <v>316</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B50"/>
+  <autoFilter ref="A1:B252"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6574,258 +8815,1268 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B251"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>113</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B92" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B96" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B98" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B99" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B101" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B102" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B103" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B104" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B106" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B107" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B108" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B109" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B110" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B111" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B115" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B116" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B117" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B118" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B119" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B120" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B121" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B126" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B133" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B134" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B138" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B139" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B141" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B143" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B144" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B146" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B147" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B148" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B149" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B150" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B151" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B152" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B153" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B154" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B155" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B156" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B157" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B158" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B159" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B160" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B161" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B162" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B163" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B164" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B165" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B166" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B167" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B168" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B169" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B170" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B171" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B172" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B173" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B174" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B175" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B176" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B177" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B178" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B179" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B180" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B181" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B182" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B183" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B184" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B185" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B186" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B187" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B188" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B189" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B190" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B191" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B192" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B193" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B194" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B195" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B196" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B197" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B198" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B199" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B200" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B201" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B202" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B203" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B204" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B205" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B206" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B207" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B208" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B209" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B210" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B211" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B212" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B213" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B214" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B215" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B216" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B217" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B218" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B219" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B220" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B221" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B222" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B223" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B224" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B225" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B226" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B227" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B228" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B229" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B230" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B231" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B232" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B233" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B234" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B235" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B236" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B237" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B238" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B239" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B240" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B241" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B242" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B243" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B244" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B245" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B246" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B247" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B248" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B249" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B250" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B251" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(store): support historical issued migration and auth guard refresh (#56)
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/issued-migration/issued_items_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/issued-migration/issued_items_migration_template.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="item_type_options">'_validations'!$A$1:$A$2</definedName>
-    <definedName name="category_name_options">'_validations'!$B$1:$B$49</definedName>
+    <definedName name="category_name_options">'_validations'!$B$1:$B$251</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="317">
   <si>
     <t>Field</t>
   </si>
@@ -47,7 +47,13 @@
     <t>employee_emp_id</t>
   </si>
   <si>
-    <t>Mandatory on first row of employee block; must exist in Employee table.</t>
+    <t>Required. Issued migration currently supports employee-based issuance only. Keep employee fields blank for continuation rows of the same employee.</t>
+  </si>
+  <si>
+    <t>Current scope</t>
+  </si>
+  <si>
+    <t>Do not provide division/vehicle/custodian values in this migration. Historical issued data is imported in employee format only.</t>
   </si>
   <si>
     <t>category_name</t>
@@ -86,6 +92,12 @@
     <t>For item_type=Asset: serial_number is preferred. asset_tag is optional (auto-generated if blank for new assets).</t>
   </si>
   <si>
+    <t>Historical asset rows without serial number</t>
+  </si>
+  <si>
+    <t>For old register data only: if serial_number and asset_tag are both blank, give the cumulative asset quantity in one row. The system will create that many issued asset records with migration placeholders internally.</t>
+  </si>
+  <si>
     <t>Consumable rows</t>
   </si>
   <si>
@@ -194,19 +206,13 @@
     <t>Personnel &amp; Administrative Division</t>
   </si>
   <si>
-    <t>Desktop</t>
-  </si>
-  <si>
-    <t>Desktop Workstation</t>
-  </si>
-  <si>
-    <t>SN-DT-0007</t>
+    <t>Laptops i5 512GB SSD 8GB RAM</t>
   </si>
   <si>
     <t>2026-02-11</t>
   </si>
   <si>
-    <t>New employee block starts</t>
+    <t>Historical asset issue without serial numbers</t>
   </si>
   <si>
     <t>LEGACY-ISSUE-EMP102-01</t>
@@ -218,54 +224,360 @@
     <t>A3 Paper Rim</t>
   </si>
   <si>
+    <t>A4 Paper Rim</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>Acid</t>
+  </si>
+  <si>
+    <t>Adapter</t>
+  </si>
+  <si>
+    <t>Adhesive Tape</t>
+  </si>
+  <si>
+    <t>Agarbati</t>
+  </si>
+  <si>
+    <t>All Pin</t>
+  </si>
+  <si>
+    <t>Almirah</t>
+  </si>
+  <si>
     <t>Attendance Register</t>
   </si>
   <si>
+    <t>Attendance register</t>
+  </si>
+  <si>
+    <t>Attendance Register (Small)</t>
+  </si>
+  <si>
+    <t>Ball Pen Achiever</t>
+  </si>
+  <si>
+    <t>Ball Pen Black</t>
+  </si>
+  <si>
+    <t>Ball Pen Blue</t>
+  </si>
+  <si>
+    <t>Ball Pen Green</t>
+  </si>
+  <si>
+    <t>Ball Pen Red</t>
+  </si>
+  <si>
+    <t>Ball Pen Uniball</t>
+  </si>
+  <si>
+    <t>Ball Pen V5</t>
+  </si>
+  <si>
+    <t>Bell</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Binder Clip  32MM</t>
+  </si>
+  <si>
+    <t>Binder Clip 25 MM</t>
+  </si>
+  <si>
+    <t>Binding Machine</t>
+  </si>
+  <si>
+    <t>Black Ball Pen</t>
+  </si>
+  <si>
     <t>Black Gel Pen</t>
   </si>
   <si>
+    <t>Black Hit</t>
+  </si>
+  <si>
+    <t>Blue Ball Pen</t>
+  </si>
+  <si>
     <t>Blue Gel Pen</t>
   </si>
   <si>
+    <t>Board Marker</t>
+  </si>
+  <si>
+    <t>Boki Chok Pump</t>
+  </si>
+  <si>
+    <t>Brown Khaki Tape</t>
+  </si>
+  <si>
+    <t>Brush Toilet</t>
+  </si>
+  <si>
+    <t>Button Folder F/S</t>
+  </si>
+  <si>
+    <t>Cables</t>
+  </si>
+  <si>
+    <t>Calculator</t>
+  </si>
+  <si>
+    <t>Camera</t>
+  </si>
+  <si>
+    <t>Candle</t>
+  </si>
+  <si>
+    <t>Carbon Paper</t>
+  </si>
+  <si>
+    <t>Cartridge</t>
+  </si>
+  <si>
+    <t>CD / OHP Marker</t>
+  </si>
+  <si>
     <t>Ceiling Fan</t>
   </si>
   <si>
+    <t>Cello Tape 1/2”</t>
+  </si>
+  <si>
+    <t>Cello Tape 2” (Big)</t>
+  </si>
+  <si>
+    <t>Chair</t>
+  </si>
+  <si>
+    <t>Chowk 15watt</t>
+  </si>
+  <si>
+    <t>Chowk Electronic 36 Watt</t>
+  </si>
+  <si>
+    <t>Clutch Pencil</t>
+  </si>
+  <si>
+    <t>CMOS Cell</t>
+  </si>
+  <si>
+    <t>Computer</t>
+  </si>
+  <si>
+    <t>Cooler</t>
+  </si>
+  <si>
+    <t>Cube Sanitary</t>
+  </si>
+  <si>
+    <t>Cup</t>
+  </si>
+  <si>
+    <t>Cutter</t>
+  </si>
+  <si>
+    <t>Dak Pad</t>
+  </si>
+  <si>
+    <t>Damper</t>
+  </si>
+  <si>
     <t>Desktop Computer i5</t>
   </si>
   <si>
     <t>Desktop Computer i7</t>
   </si>
   <si>
+    <t>Dettol pump 200ML</t>
+  </si>
+  <si>
+    <t>Diesel</t>
+  </si>
+  <si>
+    <t>Digital Podium</t>
+  </si>
+  <si>
+    <t>Dispatch Register</t>
+  </si>
+  <si>
     <t>Double Punch</t>
   </si>
   <si>
+    <t>Double Punch ( Big)</t>
+  </si>
+  <si>
+    <t>Double Punch (Small)</t>
+  </si>
+  <si>
+    <t>Drill Bits</t>
+  </si>
+  <si>
+    <t>Dry Mop Set</t>
+  </si>
+  <si>
+    <t>Dustbin Plastic (Small) with cover</t>
+  </si>
+  <si>
+    <t>Dustbin without cover</t>
+  </si>
+  <si>
+    <t>Duster</t>
+  </si>
+  <si>
+    <t>Electrical Kettle</t>
+  </si>
+  <si>
     <t>Emergency Office Purchase</t>
   </si>
   <si>
+    <t>Engagement stand</t>
+  </si>
+  <si>
+    <t>Envelop 10X145(Yellow F/Size)</t>
+  </si>
+  <si>
+    <t>Envelop 11x5 (Plain/  Without Window)</t>
+  </si>
+  <si>
+    <t>Envelop Plain(6x3)</t>
+  </si>
+  <si>
+    <t>Envelop Window  (11x4 /11x5)</t>
+  </si>
+  <si>
+    <t>Envelope Khaki A4 Size</t>
+  </si>
+  <si>
+    <t>ESI Register</t>
+  </si>
+  <si>
     <t>Exhaust Fan</t>
   </si>
   <si>
+    <t>Extension Board</t>
+  </si>
+  <si>
+    <t>External Hard disk</t>
+  </si>
+  <si>
     <t>External Hard Disk 1TB</t>
   </si>
   <si>
+    <t>Fan Regulator</t>
+  </si>
+  <si>
+    <t>Fevi Gum  (Small)</t>
+  </si>
+  <si>
+    <t>File Cover Khaki</t>
+  </si>
+  <si>
+    <t>File Cover Yellow</t>
+  </si>
+  <si>
+    <t>File Flapper</t>
+  </si>
+  <si>
+    <t>File Tag (Green)</t>
+  </si>
+  <si>
+    <t>Finger print scanner</t>
+  </si>
+  <si>
     <t>Floor Cleaner</t>
   </si>
   <si>
+    <t>Fluid / Correction Pen</t>
+  </si>
+  <si>
+    <t>Fountain Pen(Blue)</t>
+  </si>
+  <si>
+    <t>Garbage Bag(Big)</t>
+  </si>
+  <si>
+    <t>Garbage Bag(small)</t>
+  </si>
+  <si>
     <t>Garden Shovel</t>
   </si>
   <si>
+    <t>Gate pass Book</t>
+  </si>
+  <si>
+    <t>Glass</t>
+  </si>
+  <si>
+    <t>Gloves plastic</t>
+  </si>
+  <si>
+    <t>Glustic</t>
+  </si>
+  <si>
+    <t>Godrej air poket</t>
+  </si>
+  <si>
+    <t>Gum Bottle</t>
+  </si>
+  <si>
     <t>Hand Wash Liquid</t>
   </si>
   <si>
+    <t>Harpic (Blue)</t>
+  </si>
+  <si>
+    <t>Harpic (Red)</t>
+  </si>
+  <si>
+    <t>Hi-Lighter</t>
+  </si>
+  <si>
     <t>Highlighter Pen</t>
   </si>
   <si>
+    <t>Hot Case</t>
+  </si>
+  <si>
+    <t>Induction</t>
+  </si>
+  <si>
+    <t>Ink Pilot Pen</t>
+  </si>
+  <si>
+    <t>Ink Stamps</t>
+  </si>
+  <si>
     <t>Inkjet Cartridge Black</t>
   </si>
   <si>
     <t>Inkjet Cartridge Color</t>
   </si>
   <si>
+    <t>Izyol 500ML</t>
+  </si>
+  <si>
+    <t>Jharu (Soft Broom)</t>
+  </si>
+  <si>
+    <t>Jharu stick(Bans)</t>
+  </si>
+  <si>
+    <t>Jug</t>
+  </si>
+  <si>
+    <t>Key Board</t>
+  </si>
+  <si>
+    <t>Ladder</t>
+  </si>
+  <si>
     <t>Laptop i5 8GB 512GB</t>
   </si>
   <si>
@@ -275,9 +587,60 @@
     <t>LED Monitor 24 Inch</t>
   </si>
   <si>
+    <t>LED Pannel Light</t>
+  </si>
+  <si>
+    <t>LED T.V</t>
+  </si>
+  <si>
     <t>LED TV 43 Inch</t>
   </si>
   <si>
+    <t>Legal Noting Rim</t>
+  </si>
+  <si>
+    <t>Legal Rim</t>
+  </si>
+  <si>
+    <t>Lifebouy soap</t>
+  </si>
+  <si>
+    <t>Liquid Soap</t>
+  </si>
+  <si>
+    <t>Lock</t>
+  </si>
+  <si>
+    <t>Log Book</t>
+  </si>
+  <si>
+    <t>M fold tissue</t>
+  </si>
+  <si>
+    <t>MCB Box</t>
+  </si>
+  <si>
+    <t>Mobile Phone</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>MRN Book</t>
+  </si>
+  <si>
+    <t>Name Plates</t>
+  </si>
+  <si>
+    <t>Nirma surf powder</t>
+  </si>
+  <si>
+    <t>Noting Sheet</t>
+  </si>
+  <si>
+    <t>Odonil</t>
+  </si>
+  <si>
     <t>Office Car Diesel</t>
   </si>
   <si>
@@ -293,57 +656,258 @@
     <t>Office Notebook</t>
   </si>
   <si>
+    <t>Oven</t>
+  </si>
+  <si>
+    <t>Paper Weight</t>
+  </si>
+  <si>
+    <t>Pen drive</t>
+  </si>
+  <si>
     <t>Pen Drive 64GB</t>
   </si>
   <si>
+    <t>Pen stand</t>
+  </si>
+  <si>
+    <t>Pencil Cell</t>
+  </si>
+  <si>
+    <t>Pencil Ordinary</t>
+  </si>
+  <si>
+    <t>Peon Book / Acknowledgement Book</t>
+  </si>
+  <si>
     <t>Permanent Marker</t>
   </si>
   <si>
     <t>Phenyl Cleaner</t>
   </si>
   <si>
+    <t>Photocopier</t>
+  </si>
+  <si>
+    <t>Photostat paper A4 Size</t>
+  </si>
+  <si>
+    <t>Photostat Paper F/S</t>
+  </si>
+  <si>
+    <t>Phynol</t>
+  </si>
+  <si>
     <t>Pilot Blue Pen</t>
   </si>
   <si>
+    <t>Pilot Pen V7</t>
+  </si>
+  <si>
+    <t>Pin Cushion</t>
+  </si>
+  <si>
+    <t>Pochha  Simple</t>
+  </si>
+  <si>
+    <t>Poker</t>
+  </si>
+  <si>
+    <t>Pot</t>
+  </si>
+  <si>
+    <t>Printer</t>
+  </si>
+  <si>
     <t>Projector</t>
   </si>
   <si>
+    <t>PVC Pipes</t>
+  </si>
+  <si>
+    <t>Receipt Register</t>
+  </si>
+  <si>
+    <t>Refill Ordinary</t>
+  </si>
+  <si>
+    <t>Refrigerator</t>
+  </si>
+  <si>
+    <t>Register 04 Q</t>
+  </si>
+  <si>
+    <t>Register 2Q</t>
+  </si>
+  <si>
     <t>Ring Binder File</t>
   </si>
   <si>
+    <t>Room freshner</t>
+  </si>
+  <si>
+    <t>Room Heater</t>
+  </si>
+  <si>
+    <t>Router</t>
+  </si>
+  <si>
+    <t>Rubber Band</t>
+  </si>
+  <si>
+    <t>Rubber Ordinary</t>
+  </si>
+  <si>
+    <t>Scale Plastic</t>
+  </si>
+  <si>
+    <t>Scale Steel</t>
+  </si>
+  <si>
+    <t>Scanner</t>
+  </si>
+  <si>
+    <t>Scissor</t>
+  </si>
+  <si>
+    <t>Scotch brite</t>
+  </si>
+  <si>
+    <t>Screw Driver</t>
+  </si>
+  <si>
+    <t>Server</t>
+  </si>
+  <si>
+    <t>Service Book</t>
+  </si>
+  <si>
+    <t>Sharpner</t>
+  </si>
+  <si>
     <t>Single Punch</t>
   </si>
   <si>
+    <t>Sketch Pen</t>
+  </si>
+  <si>
+    <t>Slip Pad (Ordinary)</t>
+  </si>
+  <si>
+    <t>Soap Rin /Lux</t>
+  </si>
+  <si>
+    <t>Socket</t>
+  </si>
+  <si>
+    <t>Socket 15 amp</t>
+  </si>
+  <si>
+    <t>Sofa</t>
+  </si>
+  <si>
+    <t>Spiral pad</t>
+  </si>
+  <si>
     <t>Spring File</t>
   </si>
   <si>
     <t>SSD 512GB</t>
   </si>
   <si>
+    <t>Stamp for CO Proc</t>
+  </si>
+  <si>
+    <t>Stamp Pad</t>
+  </si>
+  <si>
+    <t>Stamp Pad Ink</t>
+  </si>
+  <si>
+    <t>Standing Fan</t>
+  </si>
+  <si>
     <t>Stapler</t>
   </si>
   <si>
-    <t>Stapler Pin Big</t>
+    <t>Stapler Big</t>
+  </si>
+  <si>
+    <t>Stapler pin Big</t>
   </si>
   <si>
     <t>Stapler Pin Small</t>
   </si>
   <si>
+    <t>Stapler Small</t>
+  </si>
+  <si>
     <t>Steel Almirah</t>
   </si>
   <si>
+    <t>Stick Note Pad (Yellow)</t>
+  </si>
+  <si>
     <t>Stock Register</t>
   </si>
   <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Tablets</t>
+  </si>
+  <si>
+    <t>Telephone Register</t>
+  </si>
+  <si>
+    <t>Telephone Set</t>
+  </si>
+  <si>
+    <t>Test Category 1</t>
+  </si>
+  <si>
+    <t>Test Cateogry 2</t>
+  </si>
+  <si>
+    <t>Toilet Paper roll</t>
+  </si>
+  <si>
+    <t>Toner</t>
+  </si>
+  <si>
+    <t>Tonner General</t>
+  </si>
+  <si>
+    <t>Tray</t>
+  </si>
+  <si>
+    <t>U Clip</t>
+  </si>
+  <si>
     <t>U Clip Box</t>
   </si>
   <si>
+    <t>Umbrella</t>
+  </si>
+  <si>
     <t>Uniball black Pen</t>
   </si>
   <si>
     <t>Uniball blue Pen</t>
   </si>
   <si>
+    <t>UPS</t>
+  </si>
+  <si>
+    <t>Urinal Cube</t>
+  </si>
+  <si>
+    <t>Urnal screen(Jali)</t>
+  </si>
+  <si>
     <t>V5 blue Pen</t>
   </si>
   <si>
@@ -353,13 +917,58 @@
     <t>V7 Green Pen</t>
   </si>
   <si>
+    <t>Vim Bar</t>
+  </si>
+  <si>
+    <t>Vim Liquid</t>
+  </si>
+  <si>
+    <t>Visitor Card Album</t>
+  </si>
+  <si>
     <t>Visitor Chair</t>
   </si>
   <si>
+    <t>Visitor Slip</t>
+  </si>
+  <si>
+    <t>Wall Clock</t>
+  </si>
+  <si>
+    <t>Wall Fan</t>
+  </si>
+  <si>
+    <t>Water Bottle</t>
+  </si>
+  <si>
+    <t>Water dispenser</t>
+  </si>
+  <si>
     <t>Water Hose Pipe</t>
   </si>
   <si>
+    <t>Weighing Machine</t>
+  </si>
+  <si>
+    <t>Wet Mop Refil</t>
+  </si>
+  <si>
+    <t>Wet Mop Set</t>
+  </si>
+  <si>
+    <t>White Tag</t>
+  </si>
+  <si>
+    <t>Wiper Small</t>
+  </si>
+  <si>
+    <t>Wire</t>
+  </si>
+  <si>
     <t>Wooden Cabinet</t>
+  </si>
+  <si>
+    <t>Yellow envelop A4 Size</t>
   </si>
 </sst>
 </file>
@@ -766,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -885,8 +1494,24 @@
         <v>27</v>
       </c>
     </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -917,58 +1542,58 @@
   <sheetData>
     <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -979,52 +1604,52 @@
         <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="O2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="P2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -1032,55 +1657,55 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="L3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="M3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N3">
         <v>5</v>
       </c>
       <c r="O3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="P3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="R3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1091,52 +1716,52 @@
         <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="I4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="L4" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
-      </c>
-      <c r="N4" t="s">
-        <v>43</v>
+        <v>47</v>
+      </c>
+      <c r="N4">
+        <v>30</v>
       </c>
       <c r="O4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="P4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="Q4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="R4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="5:6" x14ac:dyDescent="0.25"/>
@@ -6158,7 +6783,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B252"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -6167,10 +6792,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -6178,7 +6803,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -6186,7 +6811,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -6194,7 +6819,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -6202,7 +6827,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -6210,7 +6835,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -6218,7 +6843,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -6226,7 +6851,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -6234,7 +6859,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -6242,7 +6867,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -6250,7 +6875,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -6258,7 +6883,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -6266,7 +6891,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -6274,7 +6899,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -6282,7 +6907,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -6290,7 +6915,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -6298,7 +6923,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -6306,7 +6931,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -6314,7 +6939,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -6322,7 +6947,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -6330,7 +6955,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -6338,7 +6963,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -6346,7 +6971,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -6354,7 +6979,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -6362,7 +6987,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -6370,7 +6995,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -6378,7 +7003,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -6386,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -6394,7 +7019,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -6402,7 +7027,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -6410,7 +7035,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -6418,7 +7043,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -6426,7 +7051,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -6434,7 +7059,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -6442,7 +7067,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -6450,7 +7075,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -6458,7 +7083,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -6466,7 +7091,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -6474,7 +7099,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -6482,7 +7107,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -6490,7 +7115,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -6498,7 +7123,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -6506,7 +7131,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -6514,7 +7139,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -6522,7 +7147,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -6530,7 +7155,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -6538,7 +7163,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -6546,7 +7171,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -6554,7 +7179,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -6562,11 +7187,1627 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114">
         <v>113</v>
       </c>
+      <c r="B114" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>201</v>
+      </c>
+      <c r="B202" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>202</v>
+      </c>
+      <c r="B203" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>203</v>
+      </c>
+      <c r="B204" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>204</v>
+      </c>
+      <c r="B205" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>222</v>
+      </c>
+      <c r="B223" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>223</v>
+      </c>
+      <c r="B224" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>224</v>
+      </c>
+      <c r="B225" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>227</v>
+      </c>
+      <c r="B228" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>228</v>
+      </c>
+      <c r="B229" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>229</v>
+      </c>
+      <c r="B230" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>230</v>
+      </c>
+      <c r="B231" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>231</v>
+      </c>
+      <c r="B232" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>232</v>
+      </c>
+      <c r="B233" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>233</v>
+      </c>
+      <c r="B234" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>234</v>
+      </c>
+      <c r="B235" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>235</v>
+      </c>
+      <c r="B236" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>236</v>
+      </c>
+      <c r="B237" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>237</v>
+      </c>
+      <c r="B238" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>238</v>
+      </c>
+      <c r="B239" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A240">
+        <v>239</v>
+      </c>
+      <c r="B240" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>240</v>
+      </c>
+      <c r="B241" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>241</v>
+      </c>
+      <c r="B242" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>242</v>
+      </c>
+      <c r="B243" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>243</v>
+      </c>
+      <c r="B244" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>244</v>
+      </c>
+      <c r="B245" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>245</v>
+      </c>
+      <c r="B246" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>246</v>
+      </c>
+      <c r="B247" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>247</v>
+      </c>
+      <c r="B248" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>248</v>
+      </c>
+      <c r="B249" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>249</v>
+      </c>
+      <c r="B250" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>250</v>
+      </c>
+      <c r="B251" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>251</v>
+      </c>
+      <c r="B252" t="s">
+        <v>316</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B50"/>
+  <autoFilter ref="A1:B252"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6574,258 +8815,1268 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B251"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>113</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B92" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B96" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B98" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B99" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B101" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B102" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B103" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B104" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B106" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B107" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B108" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B109" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B110" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B111" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B115" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B116" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B117" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B118" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B119" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B120" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B121" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B126" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B133" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B134" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B138" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B139" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B141" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B143" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B144" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B146" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B147" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B148" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B149" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B150" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B151" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B152" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B153" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B154" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B155" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B156" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B157" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B158" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B159" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B160" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B161" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B162" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B163" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B164" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B165" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B166" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B167" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B168" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B169" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B170" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B171" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B172" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B173" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B174" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B175" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B176" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B177" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B178" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B179" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B180" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B181" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B182" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B183" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B184" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B185" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B186" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B187" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B188" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B189" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B190" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B191" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B192" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B193" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B194" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B195" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B196" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B197" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B198" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B199" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B200" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B201" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B202" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B203" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B204" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B205" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B206" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B207" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B208" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B209" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B210" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B211" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B212" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B213" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B214" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B215" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B216" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B217" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B218" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B219" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B220" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B221" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B222" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B223" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B224" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B225" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B226" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B227" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B228" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B229" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B230" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B231" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B232" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B233" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B234" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B235" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B236" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B237" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B238" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B239" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B240" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B241" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B242" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B243" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B244" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B245" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B246" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B247" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B248" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B249" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B250" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B251" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(migration): align location-aware imports with access control
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/issued-migration/issued_items_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/issued-migration/issued_items_migration_template.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="item_type_options">'_validations'!$A$1:$A$2</definedName>
-    <definedName name="category_name_options">'_validations'!$B$1:$B$251</definedName>
+    <definedName name="category_name_options">'_validations'!$B$1:$B$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="71">
   <si>
     <t>Field</t>
   </si>
@@ -50,6 +50,12 @@
     <t>Required. Issued migration currently supports employee-based issuance only. Keep employee fields blank for continuation rows of the same employee.</t>
   </si>
   <si>
+    <t>Location routing</t>
+  </si>
+  <si>
+    <t>Location is resolved from the employee office_location already saved in Employee master. Stock and employee must belong to the same location. Cross-location issued migration is blocked.</t>
+  </si>
+  <si>
     <t>Current scope</t>
   </si>
   <si>
@@ -221,754 +227,10 @@
     <t>sr_no</t>
   </si>
   <si>
-    <t>A3 Paper Rim</t>
-  </si>
-  <si>
-    <t>A4 Paper Rim</t>
-  </si>
-  <si>
-    <t>AC</t>
-  </si>
-  <si>
-    <t>Acid</t>
-  </si>
-  <si>
-    <t>Adapter</t>
-  </si>
-  <si>
-    <t>Adhesive Tape</t>
-  </si>
-  <si>
-    <t>Agarbati</t>
-  </si>
-  <si>
-    <t>All Pin</t>
-  </si>
-  <si>
-    <t>Almirah</t>
-  </si>
-  <si>
-    <t>Attendance Register</t>
-  </si>
-  <si>
-    <t>Attendance register</t>
-  </si>
-  <si>
-    <t>Attendance Register (Small)</t>
-  </si>
-  <si>
-    <t>Ball Pen Achiever</t>
-  </si>
-  <si>
-    <t>Ball Pen Black</t>
-  </si>
-  <si>
-    <t>Ball Pen Blue</t>
-  </si>
-  <si>
-    <t>Ball Pen Green</t>
-  </si>
-  <si>
-    <t>Ball Pen Red</t>
-  </si>
-  <si>
-    <t>Ball Pen Uniball</t>
-  </si>
-  <si>
-    <t>Ball Pen V5</t>
-  </si>
-  <si>
-    <t>Bell</t>
-  </si>
-  <si>
-    <t>Bicycle</t>
-  </si>
-  <si>
-    <t>Binder Clip  32MM</t>
-  </si>
-  <si>
-    <t>Binder Clip 25 MM</t>
-  </si>
-  <si>
-    <t>Binding Machine</t>
-  </si>
-  <si>
-    <t>Black Ball Pen</t>
-  </si>
-  <si>
-    <t>Black Gel Pen</t>
-  </si>
-  <si>
-    <t>Black Hit</t>
-  </si>
-  <si>
-    <t>Blue Ball Pen</t>
-  </si>
-  <si>
-    <t>Blue Gel Pen</t>
-  </si>
-  <si>
-    <t>Board Marker</t>
-  </si>
-  <si>
-    <t>Boki Chok Pump</t>
-  </si>
-  <si>
-    <t>Brown Khaki Tape</t>
-  </si>
-  <si>
-    <t>Brush Toilet</t>
-  </si>
-  <si>
-    <t>Button Folder F/S</t>
-  </si>
-  <si>
-    <t>Cables</t>
-  </si>
-  <si>
-    <t>Calculator</t>
-  </si>
-  <si>
-    <t>Camera</t>
-  </si>
-  <si>
-    <t>Candle</t>
-  </si>
-  <si>
-    <t>Carbon Paper</t>
-  </si>
-  <si>
-    <t>Cartridge</t>
-  </si>
-  <si>
-    <t>CD / OHP Marker</t>
-  </si>
-  <si>
-    <t>Ceiling Fan</t>
-  </si>
-  <si>
-    <t>Cello Tape 1/2”</t>
-  </si>
-  <si>
-    <t>Cello Tape 2” (Big)</t>
-  </si>
-  <si>
-    <t>Chair</t>
-  </si>
-  <si>
-    <t>Chowk 15watt</t>
-  </si>
-  <si>
-    <t>Chowk Electronic 36 Watt</t>
-  </si>
-  <si>
-    <t>Clutch Pencil</t>
-  </si>
-  <si>
-    <t>CMOS Cell</t>
-  </si>
-  <si>
-    <t>Computer</t>
-  </si>
-  <si>
-    <t>Cooler</t>
-  </si>
-  <si>
-    <t>Cube Sanitary</t>
-  </si>
-  <si>
-    <t>Cup</t>
-  </si>
-  <si>
-    <t>Cutter</t>
-  </si>
-  <si>
-    <t>Dak Pad</t>
-  </si>
-  <si>
-    <t>Damper</t>
-  </si>
-  <si>
-    <t>Desktop Computer i5</t>
-  </si>
-  <si>
-    <t>Desktop Computer i7</t>
-  </si>
-  <si>
-    <t>Dettol pump 200ML</t>
-  </si>
-  <si>
-    <t>Diesel</t>
-  </si>
-  <si>
-    <t>Digital Podium</t>
-  </si>
-  <si>
-    <t>Dispatch Register</t>
-  </si>
-  <si>
-    <t>Double Punch</t>
-  </si>
-  <si>
-    <t>Double Punch ( Big)</t>
-  </si>
-  <si>
-    <t>Double Punch (Small)</t>
-  </si>
-  <si>
-    <t>Drill Bits</t>
-  </si>
-  <si>
-    <t>Dry Mop Set</t>
-  </si>
-  <si>
-    <t>Dustbin Plastic (Small) with cover</t>
-  </si>
-  <si>
-    <t>Dustbin without cover</t>
-  </si>
-  <si>
-    <t>Duster</t>
-  </si>
-  <si>
-    <t>Electrical Kettle</t>
-  </si>
-  <si>
-    <t>Emergency Office Purchase</t>
-  </si>
-  <si>
-    <t>Engagement stand</t>
-  </si>
-  <si>
-    <t>Envelop 10X145(Yellow F/Size)</t>
-  </si>
-  <si>
-    <t>Envelop 11x5 (Plain/  Without Window)</t>
-  </si>
-  <si>
-    <t>Envelop Plain(6x3)</t>
-  </si>
-  <si>
-    <t>Envelop Window  (11x4 /11x5)</t>
-  </si>
-  <si>
-    <t>Envelope Khaki A4 Size</t>
-  </si>
-  <si>
-    <t>ESI Register</t>
-  </si>
-  <si>
-    <t>Exhaust Fan</t>
-  </si>
-  <si>
-    <t>Extension Board</t>
-  </si>
-  <si>
-    <t>External Hard disk</t>
-  </si>
-  <si>
-    <t>External Hard Disk 1TB</t>
-  </si>
-  <si>
-    <t>Fan Regulator</t>
-  </si>
-  <si>
-    <t>Fevi Gum  (Small)</t>
-  </si>
-  <si>
-    <t>File Cover Khaki</t>
-  </si>
-  <si>
-    <t>File Cover Yellow</t>
-  </si>
-  <si>
-    <t>File Flapper</t>
-  </si>
-  <si>
-    <t>File Tag (Green)</t>
-  </si>
-  <si>
-    <t>Finger print scanner</t>
-  </si>
-  <si>
-    <t>Floor Cleaner</t>
-  </si>
-  <si>
-    <t>Fluid / Correction Pen</t>
-  </si>
-  <si>
-    <t>Fountain Pen(Blue)</t>
-  </si>
-  <si>
-    <t>Garbage Bag(Big)</t>
-  </si>
-  <si>
-    <t>Garbage Bag(small)</t>
-  </si>
-  <si>
-    <t>Garden Shovel</t>
-  </si>
-  <si>
-    <t>Gate pass Book</t>
-  </si>
-  <si>
-    <t>Glass</t>
-  </si>
-  <si>
-    <t>Gloves plastic</t>
-  </si>
-  <si>
-    <t>Glustic</t>
-  </si>
-  <si>
-    <t>Godrej air poket</t>
-  </si>
-  <si>
-    <t>Gum Bottle</t>
-  </si>
-  <si>
-    <t>Hand Wash Liquid</t>
-  </si>
-  <si>
-    <t>Harpic (Blue)</t>
-  </si>
-  <si>
-    <t>Harpic (Red)</t>
-  </si>
-  <si>
-    <t>Hi-Lighter</t>
-  </si>
-  <si>
-    <t>Highlighter Pen</t>
-  </si>
-  <si>
-    <t>Hot Case</t>
-  </si>
-  <si>
-    <t>Induction</t>
-  </si>
-  <si>
-    <t>Ink Pilot Pen</t>
-  </si>
-  <si>
-    <t>Ink Stamps</t>
-  </si>
-  <si>
-    <t>Inkjet Cartridge Black</t>
-  </si>
-  <si>
-    <t>Inkjet Cartridge Color</t>
-  </si>
-  <si>
-    <t>Izyol 500ML</t>
-  </si>
-  <si>
-    <t>Jharu (Soft Broom)</t>
-  </si>
-  <si>
-    <t>Jharu stick(Bans)</t>
-  </si>
-  <si>
-    <t>Jug</t>
-  </si>
-  <si>
-    <t>Key Board</t>
-  </si>
-  <si>
-    <t>Ladder</t>
-  </si>
-  <si>
-    <t>Laptop i5 8GB 512GB</t>
-  </si>
-  <si>
-    <t>Laptop i7 16GB 1TB</t>
-  </si>
-  <si>
-    <t>LED Monitor 24 Inch</t>
-  </si>
-  <si>
-    <t>LED Pannel Light</t>
-  </si>
-  <si>
-    <t>LED T.V</t>
-  </si>
-  <si>
-    <t>LED TV 43 Inch</t>
-  </si>
-  <si>
-    <t>Legal Noting Rim</t>
-  </si>
-  <si>
-    <t>Legal Rim</t>
-  </si>
-  <si>
-    <t>Lifebouy soap</t>
-  </si>
-  <si>
-    <t>Liquid Soap</t>
-  </si>
-  <si>
-    <t>Lock</t>
-  </si>
-  <si>
-    <t>Log Book</t>
-  </si>
-  <si>
-    <t>M fold tissue</t>
-  </si>
-  <si>
-    <t>MCB Box</t>
-  </si>
-  <si>
-    <t>Mobile Phone</t>
-  </si>
-  <si>
-    <t>Mouse</t>
-  </si>
-  <si>
-    <t>MRN Book</t>
-  </si>
-  <si>
-    <t>Name Plates</t>
-  </si>
-  <si>
-    <t>Nirma surf powder</t>
-  </si>
-  <si>
-    <t>Noting Sheet</t>
-  </si>
-  <si>
-    <t>Odonil</t>
-  </si>
-  <si>
-    <t>Office Car Diesel</t>
-  </si>
-  <si>
-    <t>Office Car Petrol</t>
-  </si>
-  <si>
-    <t>Office Chair Revolving</t>
-  </si>
-  <si>
-    <t>Office File Board</t>
-  </si>
-  <si>
-    <t>Office Notebook</t>
-  </si>
-  <si>
-    <t>Oven</t>
-  </si>
-  <si>
-    <t>Paper Weight</t>
-  </si>
-  <si>
-    <t>Pen drive</t>
-  </si>
-  <si>
-    <t>Pen Drive 64GB</t>
-  </si>
-  <si>
-    <t>Pen stand</t>
-  </si>
-  <si>
-    <t>Pencil Cell</t>
-  </si>
-  <si>
-    <t>Pencil Ordinary</t>
-  </si>
-  <si>
-    <t>Peon Book / Acknowledgement Book</t>
-  </si>
-  <si>
-    <t>Permanent Marker</t>
-  </si>
-  <si>
-    <t>Phenyl Cleaner</t>
-  </si>
-  <si>
-    <t>Photocopier</t>
-  </si>
-  <si>
-    <t>Photostat paper A4 Size</t>
-  </si>
-  <si>
-    <t>Photostat Paper F/S</t>
-  </si>
-  <si>
-    <t>Phynol</t>
-  </si>
-  <si>
-    <t>Pilot Blue Pen</t>
-  </si>
-  <si>
-    <t>Pilot Pen V7</t>
-  </si>
-  <si>
-    <t>Pin Cushion</t>
-  </si>
-  <si>
-    <t>Pochha  Simple</t>
-  </si>
-  <si>
-    <t>Poker</t>
-  </si>
-  <si>
-    <t>Pot</t>
-  </si>
-  <si>
     <t>Printer</t>
   </si>
   <si>
-    <t>Projector</t>
-  </si>
-  <si>
-    <t>PVC Pipes</t>
-  </si>
-  <si>
-    <t>Receipt Register</t>
-  </si>
-  <si>
-    <t>Refill Ordinary</t>
-  </si>
-  <si>
-    <t>Refrigerator</t>
-  </si>
-  <si>
-    <t>Register 04 Q</t>
-  </si>
-  <si>
-    <t>Register 2Q</t>
-  </si>
-  <si>
-    <t>Ring Binder File</t>
-  </si>
-  <si>
-    <t>Room freshner</t>
-  </si>
-  <si>
-    <t>Room Heater</t>
-  </si>
-  <si>
-    <t>Router</t>
-  </si>
-  <si>
-    <t>Rubber Band</t>
-  </si>
-  <si>
-    <t>Rubber Ordinary</t>
-  </si>
-  <si>
-    <t>Scale Plastic</t>
-  </si>
-  <si>
-    <t>Scale Steel</t>
-  </si>
-  <si>
-    <t>Scanner</t>
-  </si>
-  <si>
-    <t>Scissor</t>
-  </si>
-  <si>
-    <t>Scotch brite</t>
-  </si>
-  <si>
-    <t>Screw Driver</t>
-  </si>
-  <si>
-    <t>Server</t>
-  </si>
-  <si>
-    <t>Service Book</t>
-  </si>
-  <si>
-    <t>Sharpner</t>
-  </si>
-  <si>
-    <t>Single Punch</t>
-  </si>
-  <si>
-    <t>Sketch Pen</t>
-  </si>
-  <si>
-    <t>Slip Pad (Ordinary)</t>
-  </si>
-  <si>
-    <t>Soap Rin /Lux</t>
-  </si>
-  <si>
-    <t>Socket</t>
-  </si>
-  <si>
-    <t>Socket 15 amp</t>
-  </si>
-  <si>
-    <t>Sofa</t>
-  </si>
-  <si>
-    <t>Spiral pad</t>
-  </si>
-  <si>
-    <t>Spring File</t>
-  </si>
-  <si>
-    <t>SSD 512GB</t>
-  </si>
-  <si>
-    <t>Stamp for CO Proc</t>
-  </si>
-  <si>
-    <t>Stamp Pad</t>
-  </si>
-  <si>
-    <t>Stamp Pad Ink</t>
-  </si>
-  <si>
-    <t>Standing Fan</t>
-  </si>
-  <si>
-    <t>Stapler</t>
-  </si>
-  <si>
-    <t>Stapler Big</t>
-  </si>
-  <si>
-    <t>Stapler pin Big</t>
-  </si>
-  <si>
-    <t>Stapler Pin Small</t>
-  </si>
-  <si>
-    <t>Stapler Small</t>
-  </si>
-  <si>
-    <t>Steel Almirah</t>
-  </si>
-  <si>
-    <t>Stick Note Pad (Yellow)</t>
-  </si>
-  <si>
-    <t>Stock Register</t>
-  </si>
-  <si>
-    <t>Switch</t>
-  </si>
-  <si>
-    <t>Table</t>
-  </si>
-  <si>
-    <t>Tablets</t>
-  </si>
-  <si>
-    <t>Telephone Register</t>
-  </si>
-  <si>
-    <t>Telephone Set</t>
-  </si>
-  <si>
-    <t>Test Category 1</t>
-  </si>
-  <si>
-    <t>Test Cateogry 2</t>
-  </si>
-  <si>
-    <t>Toilet Paper roll</t>
-  </si>
-  <si>
-    <t>Toner</t>
-  </si>
-  <si>
-    <t>Tonner General</t>
-  </si>
-  <si>
-    <t>Tray</t>
-  </si>
-  <si>
-    <t>U Clip</t>
-  </si>
-  <si>
-    <t>U Clip Box</t>
-  </si>
-  <si>
-    <t>Umbrella</t>
-  </si>
-  <si>
-    <t>Uniball black Pen</t>
-  </si>
-  <si>
-    <t>Uniball blue Pen</t>
-  </si>
-  <si>
-    <t>UPS</t>
-  </si>
-  <si>
-    <t>Urinal Cube</t>
-  </si>
-  <si>
-    <t>Urnal screen(Jali)</t>
-  </si>
-  <si>
-    <t>V5 blue Pen</t>
-  </si>
-  <si>
-    <t>V7 blue Pen</t>
-  </si>
-  <si>
-    <t>V7 Green Pen</t>
-  </si>
-  <si>
-    <t>Vim Bar</t>
-  </si>
-  <si>
-    <t>Vim Liquid</t>
-  </si>
-  <si>
-    <t>Visitor Card Album</t>
-  </si>
-  <si>
-    <t>Visitor Chair</t>
-  </si>
-  <si>
-    <t>Visitor Slip</t>
-  </si>
-  <si>
-    <t>Wall Clock</t>
-  </si>
-  <si>
-    <t>Wall Fan</t>
-  </si>
-  <si>
-    <t>Water Bottle</t>
-  </si>
-  <si>
-    <t>Water dispenser</t>
-  </si>
-  <si>
-    <t>Water Hose Pipe</t>
-  </si>
-  <si>
-    <t>Weighing Machine</t>
-  </si>
-  <si>
-    <t>Wet Mop Refil</t>
-  </si>
-  <si>
-    <t>Wet Mop Set</t>
-  </si>
-  <si>
-    <t>White Tag</t>
-  </si>
-  <si>
-    <t>Wiper Small</t>
-  </si>
-  <si>
-    <t>Wire</t>
-  </si>
-  <si>
-    <t>Wooden Cabinet</t>
-  </si>
-  <si>
-    <t>Yellow envelop A4 Size</t>
+    <t>Furniture</t>
   </si>
 </sst>
 </file>
@@ -1375,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1510,8 +772,16 @@
         <v>31</v>
       </c>
     </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B16"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1542,58 +812,58 @@
   <sheetData>
     <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -1604,52 +874,52 @@
         <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="L2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M2" t="s">
         <v>49</v>
       </c>
-      <c r="M2" t="s">
-        <v>47</v>
-      </c>
       <c r="N2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="O2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Q2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="R2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -1657,55 +927,55 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N3">
         <v>5</v>
       </c>
       <c r="O3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="P3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Q3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="R3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1716,52 +986,52 @@
         <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N4">
         <v>30</v>
       </c>
       <c r="O4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="Q4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="5:6" x14ac:dyDescent="0.25"/>
@@ -6783,7 +6053,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B252"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -6792,10 +6062,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -6803,7 +6073,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -6811,7 +6081,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -6830,1984 +6100,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>54</v>
-      </c>
-      <c r="B55" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>55</v>
-      </c>
-      <c r="B56" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63">
-        <v>62</v>
-      </c>
-      <c r="B63" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65">
-        <v>64</v>
-      </c>
-      <c r="B65" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66">
-        <v>65</v>
-      </c>
-      <c r="B66" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67">
-        <v>66</v>
-      </c>
-      <c r="B67" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68">
-        <v>67</v>
-      </c>
-      <c r="B68" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69">
-        <v>68</v>
-      </c>
-      <c r="B69" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70">
-        <v>69</v>
-      </c>
-      <c r="B70" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71">
-        <v>70</v>
-      </c>
-      <c r="B71" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72">
-        <v>71</v>
-      </c>
-      <c r="B72" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73">
-        <v>72</v>
-      </c>
-      <c r="B73" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74">
-        <v>73</v>
-      </c>
-      <c r="B74" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75">
-        <v>74</v>
-      </c>
-      <c r="B75" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76">
-        <v>75</v>
-      </c>
-      <c r="B76" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77">
-        <v>76</v>
-      </c>
-      <c r="B77" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78">
-        <v>77</v>
-      </c>
-      <c r="B78" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79">
-        <v>78</v>
-      </c>
-      <c r="B79" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80">
-        <v>79</v>
-      </c>
-      <c r="B80" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81">
-        <v>80</v>
-      </c>
-      <c r="B81" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82">
-        <v>81</v>
-      </c>
-      <c r="B82" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83">
-        <v>82</v>
-      </c>
-      <c r="B83" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84">
-        <v>83</v>
-      </c>
-      <c r="B84" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85">
-        <v>84</v>
-      </c>
-      <c r="B85" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86">
-        <v>85</v>
-      </c>
-      <c r="B86" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87">
-        <v>86</v>
-      </c>
-      <c r="B87" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88">
-        <v>87</v>
-      </c>
-      <c r="B88" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89">
-        <v>88</v>
-      </c>
-      <c r="B89" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90">
-        <v>89</v>
-      </c>
-      <c r="B90" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91">
-        <v>90</v>
-      </c>
-      <c r="B91" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92">
-        <v>91</v>
-      </c>
-      <c r="B92" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93">
-        <v>92</v>
-      </c>
-      <c r="B93" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94">
-        <v>93</v>
-      </c>
-      <c r="B94" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95">
-        <v>94</v>
-      </c>
-      <c r="B95" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96">
-        <v>95</v>
-      </c>
-      <c r="B96" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97">
-        <v>96</v>
-      </c>
-      <c r="B97" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98">
-        <v>97</v>
-      </c>
-      <c r="B98" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99">
-        <v>98</v>
-      </c>
-      <c r="B99" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100">
-        <v>99</v>
-      </c>
-      <c r="B100" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101">
-        <v>100</v>
-      </c>
-      <c r="B101" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102">
-        <v>101</v>
-      </c>
-      <c r="B102" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103">
-        <v>102</v>
-      </c>
-      <c r="B103" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104">
-        <v>103</v>
-      </c>
-      <c r="B104" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105">
-        <v>104</v>
-      </c>
-      <c r="B105" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106">
-        <v>105</v>
-      </c>
-      <c r="B106" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107">
-        <v>106</v>
-      </c>
-      <c r="B107" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108">
-        <v>107</v>
-      </c>
-      <c r="B108" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109">
-        <v>108</v>
-      </c>
-      <c r="B109" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110">
-        <v>109</v>
-      </c>
-      <c r="B110" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111">
-        <v>110</v>
-      </c>
-      <c r="B111" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112">
-        <v>111</v>
-      </c>
-      <c r="B112" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113">
-        <v>112</v>
-      </c>
-      <c r="B113" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114">
-        <v>113</v>
-      </c>
-      <c r="B114" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115">
-        <v>114</v>
-      </c>
-      <c r="B115" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116">
-        <v>115</v>
-      </c>
-      <c r="B116" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117">
-        <v>116</v>
-      </c>
-      <c r="B117" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118">
-        <v>117</v>
-      </c>
-      <c r="B118" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119">
-        <v>118</v>
-      </c>
-      <c r="B119" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120">
-        <v>119</v>
-      </c>
-      <c r="B120" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121">
-        <v>120</v>
-      </c>
-      <c r="B121" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122">
-        <v>121</v>
-      </c>
-      <c r="B122" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123">
-        <v>122</v>
-      </c>
-      <c r="B123" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124">
-        <v>123</v>
-      </c>
-      <c r="B124" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A125">
-        <v>124</v>
-      </c>
-      <c r="B125" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A126">
-        <v>125</v>
-      </c>
-      <c r="B126" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A127">
-        <v>126</v>
-      </c>
-      <c r="B127" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128">
-        <v>127</v>
-      </c>
-      <c r="B128" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129">
-        <v>128</v>
-      </c>
-      <c r="B129" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130">
-        <v>129</v>
-      </c>
-      <c r="B130" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131">
-        <v>130</v>
-      </c>
-      <c r="B131" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A132">
-        <v>131</v>
-      </c>
-      <c r="B132" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133">
-        <v>132</v>
-      </c>
-      <c r="B133" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134">
-        <v>133</v>
-      </c>
-      <c r="B134" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A135">
-        <v>134</v>
-      </c>
-      <c r="B135" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136">
-        <v>135</v>
-      </c>
-      <c r="B136" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A137">
-        <v>136</v>
-      </c>
-      <c r="B137" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A138">
-        <v>137</v>
-      </c>
-      <c r="B138" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A139">
-        <v>138</v>
-      </c>
-      <c r="B139" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A140">
-        <v>139</v>
-      </c>
-      <c r="B140" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A141">
-        <v>140</v>
-      </c>
-      <c r="B141" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A142">
-        <v>141</v>
-      </c>
-      <c r="B142" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A143">
-        <v>142</v>
-      </c>
-      <c r="B143" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A144">
-        <v>143</v>
-      </c>
-      <c r="B144" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A145">
-        <v>144</v>
-      </c>
-      <c r="B145" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A146">
-        <v>145</v>
-      </c>
-      <c r="B146" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A147">
-        <v>146</v>
-      </c>
-      <c r="B147" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A148">
-        <v>147</v>
-      </c>
-      <c r="B148" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A149">
-        <v>148</v>
-      </c>
-      <c r="B149" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A150">
-        <v>149</v>
-      </c>
-      <c r="B150" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A151">
-        <v>150</v>
-      </c>
-      <c r="B151" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A152">
-        <v>151</v>
-      </c>
-      <c r="B152" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A153">
-        <v>152</v>
-      </c>
-      <c r="B153" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A154">
-        <v>153</v>
-      </c>
-      <c r="B154" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A155">
-        <v>154</v>
-      </c>
-      <c r="B155" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A156">
-        <v>155</v>
-      </c>
-      <c r="B156" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A157">
-        <v>156</v>
-      </c>
-      <c r="B157" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A158">
-        <v>157</v>
-      </c>
-      <c r="B158" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A159">
-        <v>158</v>
-      </c>
-      <c r="B159" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A160">
-        <v>159</v>
-      </c>
-      <c r="B160" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A161">
-        <v>160</v>
-      </c>
-      <c r="B161" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A162">
-        <v>161</v>
-      </c>
-      <c r="B162" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A163">
-        <v>162</v>
-      </c>
-      <c r="B163" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A164">
-        <v>163</v>
-      </c>
-      <c r="B164" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A165">
-        <v>164</v>
-      </c>
-      <c r="B165" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A166">
-        <v>165</v>
-      </c>
-      <c r="B166" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A167">
-        <v>166</v>
-      </c>
-      <c r="B167" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A168">
-        <v>167</v>
-      </c>
-      <c r="B168" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A169">
-        <v>168</v>
-      </c>
-      <c r="B169" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A170">
-        <v>169</v>
-      </c>
-      <c r="B170" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A171">
-        <v>170</v>
-      </c>
-      <c r="B171" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A172">
-        <v>171</v>
-      </c>
-      <c r="B172" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A173">
-        <v>172</v>
-      </c>
-      <c r="B173" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A174">
-        <v>173</v>
-      </c>
-      <c r="B174" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A175">
-        <v>174</v>
-      </c>
-      <c r="B175" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A176">
-        <v>175</v>
-      </c>
-      <c r="B176" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A177">
-        <v>176</v>
-      </c>
-      <c r="B177" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A178">
-        <v>177</v>
-      </c>
-      <c r="B178" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A179">
-        <v>178</v>
-      </c>
-      <c r="B179" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A180">
-        <v>179</v>
-      </c>
-      <c r="B180" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A181">
-        <v>180</v>
-      </c>
-      <c r="B181" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A182">
-        <v>181</v>
-      </c>
-      <c r="B182" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A183">
-        <v>182</v>
-      </c>
-      <c r="B183" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A184">
-        <v>183</v>
-      </c>
-      <c r="B184" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A185">
-        <v>184</v>
-      </c>
-      <c r="B185" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A186">
-        <v>185</v>
-      </c>
-      <c r="B186" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A187">
-        <v>186</v>
-      </c>
-      <c r="B187" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A188">
-        <v>187</v>
-      </c>
-      <c r="B188" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A189">
-        <v>188</v>
-      </c>
-      <c r="B189" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A190">
-        <v>189</v>
-      </c>
-      <c r="B190" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A191">
-        <v>190</v>
-      </c>
-      <c r="B191" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A192">
-        <v>191</v>
-      </c>
-      <c r="B192" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A193">
-        <v>192</v>
-      </c>
-      <c r="B193" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A194">
-        <v>193</v>
-      </c>
-      <c r="B194" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A195">
-        <v>194</v>
-      </c>
-      <c r="B195" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A196">
-        <v>195</v>
-      </c>
-      <c r="B196" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A197">
-        <v>196</v>
-      </c>
-      <c r="B197" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A198">
-        <v>197</v>
-      </c>
-      <c r="B198" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A199">
-        <v>198</v>
-      </c>
-      <c r="B199" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A200">
-        <v>199</v>
-      </c>
-      <c r="B200" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A201">
-        <v>200</v>
-      </c>
-      <c r="B201" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A202">
-        <v>201</v>
-      </c>
-      <c r="B202" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A203">
-        <v>202</v>
-      </c>
-      <c r="B203" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A204">
-        <v>203</v>
-      </c>
-      <c r="B204" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A205">
-        <v>204</v>
-      </c>
-      <c r="B205" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A206">
-        <v>205</v>
-      </c>
-      <c r="B206" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A207">
-        <v>206</v>
-      </c>
-      <c r="B207" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A208">
-        <v>207</v>
-      </c>
-      <c r="B208" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A209">
-        <v>208</v>
-      </c>
-      <c r="B209" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A210">
-        <v>209</v>
-      </c>
-      <c r="B210" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A211">
-        <v>210</v>
-      </c>
-      <c r="B211" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A212">
-        <v>211</v>
-      </c>
-      <c r="B212" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A213">
-        <v>212</v>
-      </c>
-      <c r="B213" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A214">
-        <v>213</v>
-      </c>
-      <c r="B214" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A215">
-        <v>214</v>
-      </c>
-      <c r="B215" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A216">
-        <v>215</v>
-      </c>
-      <c r="B216" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A217">
-        <v>216</v>
-      </c>
-      <c r="B217" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A218">
-        <v>217</v>
-      </c>
-      <c r="B218" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A219">
-        <v>218</v>
-      </c>
-      <c r="B219" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A220">
-        <v>219</v>
-      </c>
-      <c r="B220" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A221">
-        <v>220</v>
-      </c>
-      <c r="B221" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A222">
-        <v>221</v>
-      </c>
-      <c r="B222" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A223">
-        <v>222</v>
-      </c>
-      <c r="B223" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A224">
-        <v>223</v>
-      </c>
-      <c r="B224" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A225">
-        <v>224</v>
-      </c>
-      <c r="B225" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A226">
-        <v>225</v>
-      </c>
-      <c r="B226" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A227">
-        <v>226</v>
-      </c>
-      <c r="B227" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A228">
-        <v>227</v>
-      </c>
-      <c r="B228" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A229">
-        <v>228</v>
-      </c>
-      <c r="B229" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A230">
-        <v>229</v>
-      </c>
-      <c r="B230" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A231">
-        <v>230</v>
-      </c>
-      <c r="B231" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A232">
-        <v>231</v>
-      </c>
-      <c r="B232" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A233">
-        <v>232</v>
-      </c>
-      <c r="B233" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A234">
-        <v>233</v>
-      </c>
-      <c r="B234" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A235">
-        <v>234</v>
-      </c>
-      <c r="B235" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A236">
-        <v>235</v>
-      </c>
-      <c r="B236" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A237">
-        <v>236</v>
-      </c>
-      <c r="B237" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A238">
-        <v>237</v>
-      </c>
-      <c r="B238" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A239">
-        <v>238</v>
-      </c>
-      <c r="B239" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A240">
-        <v>239</v>
-      </c>
-      <c r="B240" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A241">
-        <v>240</v>
-      </c>
-      <c r="B241" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A242">
-        <v>241</v>
-      </c>
-      <c r="B242" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A243">
-        <v>242</v>
-      </c>
-      <c r="B243" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A244">
-        <v>243</v>
-      </c>
-      <c r="B244" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A245">
-        <v>244</v>
-      </c>
-      <c r="B245" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A246">
-        <v>245</v>
-      </c>
-      <c r="B246" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A247">
-        <v>246</v>
-      </c>
-      <c r="B247" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A248">
-        <v>247</v>
-      </c>
-      <c r="B248" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A249">
-        <v>248</v>
-      </c>
-      <c r="B249" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A250">
-        <v>249</v>
-      </c>
-      <c r="B250" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A251">
-        <v>250</v>
-      </c>
-      <c r="B251" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A252">
-        <v>251</v>
-      </c>
-      <c r="B252" t="s">
-        <v>316</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B252"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -8815,23 +6109,23 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B251"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
@@ -8842,1241 +6136,6 @@
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B39" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B40" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B42" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B45" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B46" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B47" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B49" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B50" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B51" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B53" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B54" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B56" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B57" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B58" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B60" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B61" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B68" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B70" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B71" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B72" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B73" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B74" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B75" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B76" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B77" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B78" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B79" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B81" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B82" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B85" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B86" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B87" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B88" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B89" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B90" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B91" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B92" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B93" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B94" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B95" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B96" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B97" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B98" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B99" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B100" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B101" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B102" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B103" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B104" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B105" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B106" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B107" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B108" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B109" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B110" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B111" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B112" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B114" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B115" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B116" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B117" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B118" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B119" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B120" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B121" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B122" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B123" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B124" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B126" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B127" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B128" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B129" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B130" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B131" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B132" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B133" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B134" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B135" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B136" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B137" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B138" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B139" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B140" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B141" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B142" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B143" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B144" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B145" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B146" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B147" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B148" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B149" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B150" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B151" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B152" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B153" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B154" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B155" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B156" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B157" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B158" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B159" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B160" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B161" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B162" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B163" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B164" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B165" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B166" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B167" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B168" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B169" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B170" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B171" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B172" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B173" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B174" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B175" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B176" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B177" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B178" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B179" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B180" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B181" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B182" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B183" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B184" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B185" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B186" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B187" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B188" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B189" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B190" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B191" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B192" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B193" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B194" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B195" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B196" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B197" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B198" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B199" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B200" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B201" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B202" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B203" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B204" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B205" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B206" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B207" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B208" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B209" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B210" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B211" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B212" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B213" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B214" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B215" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B216" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B217" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B218" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B219" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B220" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B221" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B222" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B223" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B224" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B225" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B226" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B227" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B228" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B229" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B230" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B231" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B232" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B233" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B234" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B235" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B236" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B237" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B238" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B239" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B240" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B241" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B242" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B243" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B244" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B245" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B246" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B247" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B248" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B249" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B250" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B251" t="s">
-        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>